<commit_message>
Configurações iniciais do projeto
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uipath-my.sharepoint.com/personal/alexandra_veizu_uipath_com/Documents/Documents/Projects/REFrameworkNET5/StudioTemplates/REFramework/contentFiles/any/any/pt2/VisualBasic/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://suzano-my.sharepoint.com/personal/julianobs_suzano_com_br/Documents/Area Dev/GitHub/UiPath/ExtracaoFaturasImgComIA/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8C54E24-BA5C-4BF9-8DAB-2778512EC11B}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1677B9F0-E625-44EB-9018-6A2D0A33E04B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="56">
   <si>
     <t>Name</t>
   </si>
@@ -160,6 +160,39 @@
   </si>
   <si>
     <t>ProcessABCQueue</t>
+  </si>
+  <si>
+    <t>url_Request</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>Shared</t>
+  </si>
+  <si>
+    <t>Url de chamada API</t>
+  </si>
+  <si>
+    <t>modelo</t>
+  </si>
+  <si>
+    <t>Modelo da IA a ser usado</t>
+  </si>
+  <si>
+    <t>Modelo</t>
+  </si>
+  <si>
+    <t>api_key</t>
+  </si>
+  <si>
+    <t>ApiKey</t>
+  </si>
+  <si>
+    <t>Chave de API Gemini</t>
+  </si>
+  <si>
+    <t>NaoSeAplica</t>
   </si>
 </sst>
 </file>
@@ -212,10 +245,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -239,9 +272,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -279,7 +312,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -385,7 +418,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -527,7 +560,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -536,12 +569,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z998"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5546875" customWidth="1"/>
+    <col min="1" max="1" width="43.5703125" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col min="3" max="3" width="81.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -589,17 +622,19 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="C3" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="28.8">
+    <row r="5" spans="1:26" ht="30">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -610,7 +645,17 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
+        <v>54</v>
+      </c>
+    </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1613,12 +1658,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col min="3" max="3" width="75.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1655,7 +1700,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="28.8">
+    <row r="2" spans="1:26" ht="30">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1666,7 +1711,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -1780,7 +1825,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="28.8">
+    <row r="17" spans="1:3" ht="45">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2771,12 +2816,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.88671875" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" customWidth="1"/>
-    <col min="3" max="3" width="60.33203125" customWidth="1"/>
-    <col min="4" max="26" width="65.44140625" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="3" max="3" width="60.28515625" customWidth="1"/>
+    <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -2815,8 +2860,34 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="2" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
+        <v>50</v>
+      </c>
+    </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Confugaração para salvar dados em excel
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://suzano-my.sharepoint.com/personal/julianobs_suzano_com_br/Documents/Area Dev/GitHub/UiPath/ExtracaoFaturasImgComIA/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1677B9F0-E625-44EB-9018-6A2D0A33E04B}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D356C666-A615-4D97-9AA4-62A2ED4E17F1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="56">
   <si>
     <t>Name</t>
   </si>
@@ -183,9 +183,6 @@
     <t>Modelo</t>
   </si>
   <si>
-    <t>api_key</t>
-  </si>
-  <si>
     <t>ApiKey</t>
   </si>
   <si>
@@ -193,6 +190,9 @@
   </si>
   <si>
     <t>NaoSeAplica</t>
+  </si>
+  <si>
+    <t>Gemini_API_Key</t>
   </si>
 </sst>
 </file>
@@ -269,6 +269,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -568,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z998"/>
+  <dimension ref="A1:Z997"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -627,7 +631,7 @@
         <v>31</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>32</v>
@@ -645,17 +649,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" t="s">
-        <v>54</v>
-      </c>
-    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1647,7 +1641,6 @@
     <row r="995" ht="14.25" customHeight="1"/>
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2888,7 +2881,20 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" t="s">
+        <v>53</v>
+      </c>
+    </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>